<commit_message>
muestras y pruebas con la esp32
</commit_message>
<xml_diff>
--- a/CuentasProyecto.xlsx
+++ b/CuentasProyecto.xlsx
@@ -1,26 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carje\Documents\U\Diseño\Proyecto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://correouisedu-my.sharepoint.com/personal/gerson2192987_correo_uis_edu_co/Documents/Documents/2025-1/DISEÑO DE CIRCUITOS ELECTRONICOS/Project_Electronic_System_Design_B1/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20F3C4A-BFE0-4B75-B90D-D2A2AA429ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A5F64801-BEB3-4D43-87F9-B20DBC046FC1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{A5F64801-BEB3-4D43-87F9-B20DBC046FC1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja1 (2)" sheetId="2" r:id="rId2"/>
     <sheet name="V3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -362,7 +373,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -375,27 +386,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -404,84 +394,84 @@
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -503,9 +493,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -543,7 +533,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -649,7 +639,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -791,7 +781,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -806,25 +796,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
       <c r="E3" s="2" t="s">
         <v>2</v>
       </c>
@@ -834,25 +824,25 @@
       <c r="G3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="16"/>
-      <c r="J3" s="22" t="s">
+      <c r="I3" s="17"/>
+      <c r="J3" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="22"/>
-      <c r="L3" s="24" t="s">
+      <c r="K3" s="16"/>
+      <c r="L3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="24"/>
+      <c r="M3" s="14"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
       <c r="E4" s="3">
         <v>2</v>
       </c>
@@ -862,27 +852,27 @@
       <c r="G4" s="4">
         <v>33272</v>
       </c>
-      <c r="H4" s="17">
+      <c r="H4" s="18">
         <f>G4*F4</f>
         <v>33272</v>
       </c>
-      <c r="I4" s="17"/>
-      <c r="J4" s="21">
+      <c r="I4" s="18"/>
+      <c r="J4" s="15">
         <f>G4*E4</f>
         <v>66544</v>
       </c>
-      <c r="K4" s="22"/>
-      <c r="L4" s="23" t="s">
+      <c r="K4" s="16"/>
+      <c r="L4" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="M4" s="24"/>
+      <c r="M4" s="14"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
       <c r="E5" s="3">
         <v>1</v>
       </c>
@@ -892,27 +882,27 @@
       <c r="G5" s="5">
         <v>22045</v>
       </c>
-      <c r="H5" s="17">
+      <c r="H5" s="18">
         <f t="shared" ref="H5:H8" si="0">G5*F5</f>
         <v>22045</v>
       </c>
-      <c r="I5" s="17"/>
-      <c r="J5" s="21">
+      <c r="I5" s="18"/>
+      <c r="J5" s="15">
         <f t="shared" ref="J5:J8" si="1">G5*E5</f>
         <v>22045</v>
       </c>
-      <c r="K5" s="22"/>
-      <c r="L5" s="23" t="s">
+      <c r="K5" s="16"/>
+      <c r="L5" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="M5" s="24"/>
+      <c r="M5" s="14"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
       <c r="E6" s="3">
         <v>4</v>
       </c>
@@ -922,27 +912,27 @@
       <c r="G6" s="5">
         <v>1327</v>
       </c>
-      <c r="H6" s="17">
+      <c r="H6" s="18">
         <f>G6*F6</f>
         <v>2654</v>
       </c>
-      <c r="I6" s="17"/>
-      <c r="J6" s="21">
+      <c r="I6" s="18"/>
+      <c r="J6" s="15">
         <f>G6*E6</f>
         <v>5308</v>
       </c>
-      <c r="K6" s="22"/>
-      <c r="L6" s="23" t="s">
+      <c r="K6" s="16"/>
+      <c r="L6" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="24"/>
+      <c r="M6" s="14"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
       <c r="E7" s="3">
         <v>6</v>
       </c>
@@ -952,30 +942,30 @@
       <c r="G7" s="5">
         <v>1633</v>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="18">
         <f>G7*F7</f>
         <v>8165</v>
       </c>
-      <c r="I7" s="17"/>
-      <c r="J7" s="21">
+      <c r="I7" s="18"/>
+      <c r="J7" s="15">
         <f>G7*E7</f>
         <v>9798</v>
       </c>
-      <c r="K7" s="22"/>
-      <c r="L7" s="23" t="s">
+      <c r="K7" s="16"/>
+      <c r="L7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="24"/>
+      <c r="M7" s="14"/>
       <c r="N7" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
       <c r="E8" s="3">
         <v>4</v>
       </c>
@@ -985,30 +975,30 @@
       <c r="G8" s="5">
         <v>2143</v>
       </c>
-      <c r="H8" s="17">
+      <c r="H8" s="18">
         <f t="shared" si="0"/>
         <v>4286</v>
       </c>
-      <c r="I8" s="17"/>
-      <c r="J8" s="21">
+      <c r="I8" s="18"/>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
         <v>8572</v>
       </c>
-      <c r="K8" s="22"/>
-      <c r="L8" s="23" t="s">
+      <c r="K8" s="16"/>
+      <c r="L8" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="M8" s="24"/>
+      <c r="M8" s="14"/>
       <c r="N8" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
       <c r="E9" s="3">
         <v>5</v>
       </c>
@@ -1018,25 +1008,25 @@
       <c r="G9" s="5">
         <v>2000</v>
       </c>
-      <c r="H9" s="17">
+      <c r="H9" s="18">
         <f t="shared" ref="H9:H11" si="2">G9*F9</f>
         <v>8000</v>
       </c>
-      <c r="I9" s="17"/>
-      <c r="J9" s="21">
+      <c r="I9" s="18"/>
+      <c r="J9" s="15">
         <f t="shared" ref="J9:J10" si="3">G9*E9</f>
         <v>10000</v>
       </c>
-      <c r="K9" s="22"/>
-      <c r="L9" s="24"/>
-      <c r="M9" s="24"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="14"/>
+      <c r="M9" s="14"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
       <c r="E10" s="3">
         <v>5</v>
       </c>
@@ -1046,28 +1036,28 @@
       <c r="G10" s="5">
         <v>1000</v>
       </c>
-      <c r="H10" s="17">
+      <c r="H10" s="18">
         <f t="shared" si="2"/>
         <v>4000</v>
       </c>
-      <c r="I10" s="17"/>
-      <c r="J10" s="21">
+      <c r="I10" s="18"/>
+      <c r="J10" s="15">
         <f t="shared" si="3"/>
         <v>5000</v>
       </c>
-      <c r="K10" s="22"/>
-      <c r="L10" s="24"/>
-      <c r="M10" s="24"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
       <c r="E11" s="3">
         <v>3</v>
       </c>
@@ -1077,23 +1067,23 @@
       <c r="G11" s="5">
         <v>5000</v>
       </c>
-      <c r="H11" s="17">
+      <c r="H11" s="18">
         <f t="shared" si="2"/>
         <v>10000</v>
       </c>
-      <c r="I11" s="17"/>
-      <c r="J11" s="21">
+      <c r="I11" s="18"/>
+      <c r="J11" s="15">
         <f t="shared" ref="J11:J14" si="4">G11*E11</f>
         <v>15000</v>
       </c>
-      <c r="K11" s="22"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="24"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="14"/>
+      <c r="M11" s="14"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
       <c r="E12" s="3">
         <v>0</v>
       </c>
@@ -1103,23 +1093,23 @@
       <c r="G12" s="5">
         <v>5000</v>
       </c>
-      <c r="H12" s="17">
+      <c r="H12" s="18">
         <f t="shared" ref="H12:H14" si="5">G12*F12</f>
         <v>0</v>
       </c>
-      <c r="I12" s="17"/>
-      <c r="J12" s="21">
+      <c r="I12" s="18"/>
+      <c r="J12" s="15">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="K12" s="22"/>
-      <c r="L12" s="24"/>
-      <c r="M12" s="24"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
       <c r="E13" s="3">
         <v>0</v>
       </c>
@@ -1129,21 +1119,21 @@
       <c r="G13" s="5">
         <v>5000</v>
       </c>
-      <c r="H13" s="17">
+      <c r="H13" s="18">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I13" s="17"/>
-      <c r="J13" s="21">
+      <c r="I13" s="18"/>
+      <c r="J13" s="15">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="K13" s="22"/>
+      <c r="K13" s="16"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
       <c r="E14" s="3">
         <v>0</v>
       </c>
@@ -1153,58 +1143,80 @@
       <c r="G14" s="5">
         <v>5000</v>
       </c>
-      <c r="H14" s="17">
+      <c r="H14" s="18">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I14" s="17"/>
-      <c r="J14" s="21">
+      <c r="I14" s="18"/>
+      <c r="J14" s="15">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="K14" s="22"/>
+      <c r="K14" s="16"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="21">
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="15">
         <f>SUM(H4:I14)</f>
         <v>92422</v>
       </c>
-      <c r="I15" s="22"/>
-      <c r="J15" s="21">
+      <c r="I15" s="16"/>
+      <c r="J15" s="15">
         <f>SUM(J4:K14)</f>
         <v>142267</v>
       </c>
-      <c r="K15" s="22"/>
+      <c r="K15" s="16"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H16" s="21">
+      <c r="H16" s="15">
         <f>H15/4</f>
         <v>23105.5</v>
       </c>
-      <c r="I16" s="22"/>
-      <c r="J16" s="21">
+      <c r="I16" s="16"/>
+      <c r="J16" s="15">
         <f>J15/4</f>
         <v>35566.75</v>
       </c>
-      <c r="K16" s="22"/>
+      <c r="K16" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="J16:K16"/>
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="H3:I3"/>
@@ -1218,38 +1230,16 @@
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="H16:I16"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="L10:M10"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
@@ -1275,25 +1265,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
       <c r="E3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1303,186 +1293,186 @@
       <c r="G3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="16"/>
-      <c r="J3" s="22" t="s">
+      <c r="I3" s="17"/>
+      <c r="J3" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="22"/>
-      <c r="L3" s="24" t="s">
+      <c r="K3" s="16"/>
+      <c r="L3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="24"/>
+      <c r="M3" s="14"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="6">
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="3">
         <v>2</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="3">
         <v>1</v>
       </c>
       <c r="G4" s="4">
         <v>33272</v>
       </c>
-      <c r="H4" s="17">
+      <c r="H4" s="18">
         <f>G4*F4</f>
         <v>33272</v>
       </c>
-      <c r="I4" s="17"/>
-      <c r="J4" s="21">
+      <c r="I4" s="18"/>
+      <c r="J4" s="15">
         <f>G4*E4</f>
         <v>66544</v>
       </c>
-      <c r="K4" s="22"/>
-      <c r="L4" s="23" t="s">
+      <c r="K4" s="16"/>
+      <c r="L4" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="M4" s="24"/>
+      <c r="M4" s="14"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="6">
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="3">
         <v>1</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="3">
         <v>1</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="5">
         <v>22045</v>
       </c>
-      <c r="H5" s="17">
+      <c r="H5" s="18">
         <f t="shared" ref="H5:H8" si="0">G5*F5</f>
         <v>22045</v>
       </c>
-      <c r="I5" s="17"/>
-      <c r="J5" s="21">
+      <c r="I5" s="18"/>
+      <c r="J5" s="15">
         <f t="shared" ref="J5:J8" si="1">G5*E5</f>
         <v>22045</v>
       </c>
-      <c r="K5" s="22"/>
-      <c r="L5" s="23" t="s">
+      <c r="K5" s="16"/>
+      <c r="L5" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="M5" s="24"/>
+      <c r="M5" s="14"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="6">
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="3">
         <v>2</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="3">
         <v>1</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="5">
         <v>1327</v>
       </c>
-      <c r="H6" s="17">
+      <c r="H6" s="18">
         <f>G6*F6</f>
         <v>1327</v>
       </c>
-      <c r="I6" s="17"/>
-      <c r="J6" s="21">
+      <c r="I6" s="18"/>
+      <c r="J6" s="15">
         <f>G6*E6</f>
         <v>2654</v>
       </c>
-      <c r="K6" s="22"/>
-      <c r="L6" s="23" t="s">
+      <c r="K6" s="16"/>
+      <c r="L6" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="24"/>
+      <c r="M6" s="14"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="8">
+      <c r="C7" s="21"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="3">
         <v>2</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="3">
         <v>1</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="5">
         <v>1480</v>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="18">
         <f>G7*F7</f>
         <v>1480</v>
       </c>
-      <c r="I7" s="17"/>
-      <c r="J7" s="21">
+      <c r="I7" s="18"/>
+      <c r="J7" s="15">
         <f>G7*E7</f>
         <v>2960</v>
       </c>
-      <c r="K7" s="22"/>
-      <c r="L7" s="23" t="s">
+      <c r="K7" s="16"/>
+      <c r="L7" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="M7" s="24"/>
+      <c r="M7" s="14"/>
       <c r="N7" s="1"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="19"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="8">
+      <c r="C8" s="21"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="3">
         <v>5</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="3">
         <v>4</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="5">
         <v>1021</v>
       </c>
-      <c r="H8" s="17">
+      <c r="H8" s="18">
         <f t="shared" si="0"/>
         <v>4084</v>
       </c>
-      <c r="I8" s="17"/>
-      <c r="J8" s="21">
+      <c r="I8" s="18"/>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
         <v>5105</v>
       </c>
-      <c r="K8" s="22"/>
-      <c r="L8" s="23" t="s">
+      <c r="K8" s="16"/>
+      <c r="L8" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="M8" s="24"/>
+      <c r="M8" s="14"/>
       <c r="N8" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="8">
+      <c r="C9" s="21"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="3">
         <v>3</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="3">
         <v>2</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="5">
         <v>2909</v>
       </c>
       <c r="H9" s="25">
@@ -1490,29 +1480,29 @@
         <v>5818</v>
       </c>
       <c r="I9" s="26"/>
-      <c r="J9" s="27">
+      <c r="J9" s="23">
         <f t="shared" ref="J9:J18" si="3">G9*E9</f>
         <v>8727</v>
       </c>
-      <c r="K9" s="28"/>
-      <c r="L9" s="23" t="s">
+      <c r="K9" s="24"/>
+      <c r="L9" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="M9" s="24"/>
+      <c r="M9" s="14"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="8">
+      <c r="C10" s="21"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="3">
         <v>5</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="3">
         <v>4</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="5">
         <v>510</v>
       </c>
       <c r="H10" s="25">
@@ -1520,29 +1510,29 @@
         <v>2040</v>
       </c>
       <c r="I10" s="26"/>
-      <c r="J10" s="27">
+      <c r="J10" s="23">
         <f t="shared" si="3"/>
         <v>2550</v>
       </c>
-      <c r="K10" s="28"/>
-      <c r="L10" s="23" t="s">
+      <c r="K10" s="24"/>
+      <c r="L10" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="M10" s="24"/>
+      <c r="M10" s="14"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="8">
+      <c r="C11" s="21"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="3">
         <v>5</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="3">
         <v>4</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="5">
         <v>561</v>
       </c>
       <c r="H11" s="25">
@@ -1550,29 +1540,29 @@
         <v>2244</v>
       </c>
       <c r="I11" s="26"/>
-      <c r="J11" s="27">
+      <c r="J11" s="23">
         <f t="shared" si="3"/>
         <v>2805</v>
       </c>
-      <c r="K11" s="28"/>
-      <c r="L11" s="23" t="s">
+      <c r="K11" s="24"/>
+      <c r="L11" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="M11" s="24"/>
+      <c r="M11" s="14"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="8">
+      <c r="C12" s="21"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="3">
         <v>2</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="3">
         <v>2</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="5">
         <v>1684</v>
       </c>
       <c r="H12" s="25">
@@ -1580,29 +1570,29 @@
         <v>3368</v>
       </c>
       <c r="I12" s="26"/>
-      <c r="J12" s="27">
+      <c r="J12" s="23">
         <f t="shared" si="3"/>
         <v>3368</v>
       </c>
-      <c r="K12" s="28"/>
-      <c r="L12" s="23" t="s">
+      <c r="K12" s="24"/>
+      <c r="L12" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="M12" s="24"/>
+      <c r="M12" s="14"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="8">
+      <c r="C13" s="21"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="3">
         <v>0</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="3">
         <v>0</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="5">
         <v>1072</v>
       </c>
       <c r="H13" s="25">
@@ -1610,28 +1600,28 @@
         <v>0</v>
       </c>
       <c r="I13" s="26"/>
-      <c r="J13" s="27">
+      <c r="J13" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K13" s="28"/>
+      <c r="K13" s="24"/>
       <c r="L13" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="8">
+      <c r="C14" s="21"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="3">
         <v>8</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="3">
         <v>6</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="5">
         <v>510</v>
       </c>
       <c r="H14" s="25">
@@ -1639,28 +1629,28 @@
         <v>3060</v>
       </c>
       <c r="I14" s="26"/>
-      <c r="J14" s="27">
+      <c r="J14" s="23">
         <f t="shared" si="3"/>
         <v>4080</v>
       </c>
-      <c r="K14" s="28"/>
+      <c r="K14" s="24"/>
       <c r="L14" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="8">
+      <c r="C15" s="21"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="3">
         <v>3</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="3">
         <v>2</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="5">
         <v>868</v>
       </c>
       <c r="H15" s="25">
@@ -1668,11 +1658,11 @@
         <v>1736</v>
       </c>
       <c r="I15" s="26"/>
-      <c r="J15" s="27">
+      <c r="J15" s="23">
         <f t="shared" si="3"/>
         <v>2604</v>
       </c>
-      <c r="K15" s="28"/>
+      <c r="K15" s="24"/>
       <c r="L15" s="1" t="s">
         <v>43</v>
       </c>
@@ -1681,18 +1671,18 @@
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="8">
+      <c r="C16" s="21"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="3">
         <v>2</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="3">
         <v>1</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="5">
         <v>500</v>
       </c>
       <c r="H16" s="25">
@@ -1700,28 +1690,28 @@
         <v>500</v>
       </c>
       <c r="I16" s="26"/>
-      <c r="J16" s="27">
+      <c r="J16" s="23">
         <f t="shared" si="3"/>
         <v>1000</v>
       </c>
-      <c r="K16" s="28"/>
+      <c r="K16" s="24"/>
       <c r="L16" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="8">
+      <c r="C17" s="21"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="3">
         <v>2</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="3">
         <v>1</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="5">
         <v>1582</v>
       </c>
       <c r="H17" s="25">
@@ -1729,26 +1719,26 @@
         <v>1582</v>
       </c>
       <c r="I17" s="26"/>
-      <c r="J17" s="27">
+      <c r="J17" s="23">
         <f t="shared" si="3"/>
         <v>3164</v>
       </c>
-      <c r="K17" s="28"/>
+      <c r="K17" s="24"/>
       <c r="L17" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B18" s="18"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="8">
+      <c r="B18" s="20"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="3">
         <v>0</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="3">
         <v>0</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="5">
         <v>0</v>
       </c>
       <c r="H18" s="25">
@@ -1756,70 +1746,89 @@
         <v>0</v>
       </c>
       <c r="I18" s="26"/>
-      <c r="J18" s="27">
+      <c r="J18" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K18" s="28"/>
+      <c r="K18" s="24"/>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="21">
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="15">
         <f>SUM(H4:I17)</f>
         <v>82556</v>
       </c>
-      <c r="I19" s="22"/>
-      <c r="J19" s="21">
+      <c r="I19" s="16"/>
+      <c r="J19" s="15">
         <f>SUM(J4:K18)</f>
         <v>127606</v>
       </c>
-      <c r="K19" s="22"/>
+      <c r="K19" s="16"/>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="H20" s="27">
+      <c r="H20" s="23">
         <f>H19/4</f>
         <v>20639</v>
       </c>
-      <c r="I20" s="28"/>
-      <c r="J20" s="27">
+      <c r="I20" s="24"/>
+      <c r="J20" s="23">
         <f>J19/4</f>
         <v>31901.5</v>
       </c>
-      <c r="K20" s="28"/>
+      <c r="K20" s="24"/>
       <c r="M20" s="1"/>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B22" s="18"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="9"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="65">
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="L3:M3"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="J4:K4"/>
@@ -1836,40 +1845,21 @@
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="H19:I19"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="L4" r:id="rId1" xr:uid="{334269ED-F581-447D-892B-ED2CD5DB0073}"/>
@@ -1902,214 +1892,214 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="20"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="22"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="11" t="s">
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16" t="s">
+      <c r="I3" s="17"/>
+      <c r="J3" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="16"/>
-      <c r="L3" s="24" t="s">
+      <c r="K3" s="17"/>
+      <c r="L3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="24"/>
+      <c r="M3" s="14"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="11">
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="3">
         <v>2</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="3">
         <v>1</v>
       </c>
-      <c r="G4" s="15">
+      <c r="G4" s="8">
         <v>33450</v>
       </c>
-      <c r="H4" s="17">
+      <c r="H4" s="18">
         <f>G4*F4</f>
         <v>33450</v>
       </c>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17">
+      <c r="I4" s="18"/>
+      <c r="J4" s="18">
         <f>G4*E4</f>
         <v>66900</v>
       </c>
-      <c r="K4" s="16"/>
-      <c r="L4" s="23" t="s">
+      <c r="K4" s="17"/>
+      <c r="L4" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="M4" s="24"/>
+      <c r="M4" s="14"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="11">
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="3">
         <v>2</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="3">
         <v>1</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="5">
         <v>20208</v>
       </c>
-      <c r="H5" s="17">
+      <c r="H5" s="18">
         <f t="shared" ref="H5:H12" si="0">G5*F5</f>
         <v>20208</v>
       </c>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17">
+      <c r="I5" s="18"/>
+      <c r="J5" s="18">
         <f t="shared" ref="J5:J12" si="1">G5*E5</f>
         <v>40416</v>
       </c>
-      <c r="K5" s="16"/>
-      <c r="L5" s="23" t="s">
+      <c r="K5" s="17"/>
+      <c r="L5" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="M5" s="24"/>
+      <c r="M5" s="14"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="11">
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="3">
         <v>2</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="3">
         <v>1</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="5">
         <v>1327</v>
       </c>
-      <c r="H6" s="17">
+      <c r="H6" s="18">
         <f>G6*F6</f>
         <v>1327</v>
       </c>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17">
+      <c r="I6" s="18"/>
+      <c r="J6" s="18">
         <f>G6*E6</f>
         <v>2654</v>
       </c>
-      <c r="K6" s="16"/>
-      <c r="L6" s="23" t="s">
+      <c r="K6" s="17"/>
+      <c r="L6" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="24"/>
+      <c r="M6" s="14"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="11">
+      <c r="C7" s="21"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="3">
         <v>2</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="3">
         <v>1</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="5">
         <v>18116</v>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="18">
         <f>G7*F7</f>
         <v>18116</v>
       </c>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17">
+      <c r="I7" s="18"/>
+      <c r="J7" s="18">
         <f>G7*E7</f>
         <v>36232</v>
       </c>
-      <c r="K7" s="16"/>
-      <c r="L7" s="23" t="s">
+      <c r="K7" s="17"/>
+      <c r="L7" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="M7" s="24"/>
+      <c r="M7" s="14"/>
       <c r="N7" s="1"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="19"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="11">
+      <c r="C8" s="21"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="3">
         <v>3</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="3">
         <v>2</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G8" s="5">
         <v>1021</v>
       </c>
-      <c r="H8" s="17">
+      <c r="H8" s="18">
         <f t="shared" si="0"/>
         <v>2042</v>
       </c>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17">
+      <c r="I8" s="18"/>
+      <c r="J8" s="18">
         <f t="shared" si="1"/>
         <v>3063</v>
       </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="23" t="s">
+      <c r="K8" s="17"/>
+      <c r="L8" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="M8" s="24"/>
+      <c r="M8" s="14"/>
       <c r="N8" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="11">
+      <c r="C9" s="21"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="3">
         <v>3</v>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="3">
         <v>2</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="5">
         <v>2909</v>
       </c>
       <c r="H9" s="25">
@@ -2122,24 +2112,24 @@
         <v>8727</v>
       </c>
       <c r="K9" s="26"/>
-      <c r="L9" s="23" t="s">
+      <c r="L9" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="M9" s="24"/>
+      <c r="M9" s="14"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="11">
+      <c r="C10" s="21"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="3">
         <v>6</v>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="3">
         <v>7</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="5">
         <v>510</v>
       </c>
       <c r="H10" s="25">
@@ -2152,24 +2142,24 @@
         <v>3060</v>
       </c>
       <c r="K10" s="26"/>
-      <c r="L10" s="23" t="s">
+      <c r="L10" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="M10" s="24"/>
+      <c r="M10" s="14"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="11">
+      <c r="C11" s="21"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="3">
         <v>6</v>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="3">
         <v>5</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="5">
         <v>561</v>
       </c>
       <c r="H11" s="25">
@@ -2182,24 +2172,24 @@
         <v>3366</v>
       </c>
       <c r="K11" s="26"/>
-      <c r="L11" s="23" t="s">
+      <c r="L11" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="M11" s="24"/>
+      <c r="M11" s="14"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="11">
+      <c r="C12" s="21"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="3">
         <v>2</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="3">
         <v>2</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="5">
         <v>1684</v>
       </c>
       <c r="H12" s="25">
@@ -2212,24 +2202,24 @@
         <v>3368</v>
       </c>
       <c r="K12" s="26"/>
-      <c r="L12" s="23" t="s">
+      <c r="L12" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="M12" s="24"/>
+      <c r="M12" s="14"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="11">
+      <c r="C13" s="21"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="3">
         <v>6</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="3">
         <v>5</v>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="5">
         <v>510</v>
       </c>
       <c r="H13" s="25">
@@ -2247,46 +2237,46 @@
       </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="17">
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="18">
         <f>SUM(H4:I13)</f>
         <v>93254</v>
       </c>
-      <c r="I14" s="16"/>
-      <c r="J14" s="17">
+      <c r="I14" s="17"/>
+      <c r="J14" s="18">
         <f>SUM(J4:K13)</f>
         <v>170846</v>
       </c>
-      <c r="K14" s="16"/>
+      <c r="K14" s="17"/>
     </row>
     <row r="15" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="22">
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="16">
         <v>4</v>
       </c>
-      <c r="G15" s="22"/>
-      <c r="H15" s="32">
+      <c r="G15" s="16"/>
+      <c r="H15" s="29">
         <f>H14/4</f>
         <v>23313.5</v>
       </c>
-      <c r="I15" s="32"/>
-      <c r="J15" s="27">
+      <c r="I15" s="29"/>
+      <c r="J15" s="23">
         <f>J14/4</f>
         <v>42711.5</v>
       </c>
-      <c r="K15" s="28"/>
+      <c r="K15" s="24"/>
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
@@ -2294,151 +2284,165 @@
         <v>52</v>
       </c>
       <c r="C16" s="26"/>
-      <c r="D16" s="39">
+      <c r="D16" s="13">
         <v>82000</v>
       </c>
-      <c r="E16" s="30"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="25" t="s">
         <v>51</v>
       </c>
       <c r="G16" s="26"/>
-      <c r="H16" s="38">
+      <c r="H16" s="35">
         <f>H14-D16</f>
         <v>11254</v>
       </c>
-      <c r="I16" s="38"/>
-      <c r="J16" s="27">
+      <c r="I16" s="35"/>
+      <c r="J16" s="23">
         <f>H16/F15</f>
         <v>2813.5</v>
       </c>
-      <c r="K16" s="28"/>
+      <c r="K16" s="24"/>
       <c r="L16" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="17" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="22">
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="16">
         <v>4</v>
       </c>
-      <c r="G17" s="22"/>
-      <c r="H17" s="31">
+      <c r="G17" s="16"/>
+      <c r="H17" s="34">
         <f>H16/F15</f>
         <v>2813.5</v>
       </c>
-      <c r="I17" s="31"/>
-      <c r="J17" s="27">
+      <c r="I17" s="34"/>
+      <c r="J17" s="23">
         <f>H17</f>
         <v>2813.5</v>
       </c>
-      <c r="K17" s="28"/>
+      <c r="K17" s="24"/>
       <c r="L17" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17">
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18">
         <v>250000</v>
       </c>
-      <c r="I18" s="17"/>
-      <c r="J18" s="13">
+      <c r="I18" s="18"/>
+      <c r="J18" s="6">
         <f>G18*E18</f>
         <v>0</v>
       </c>
-      <c r="K18" s="14"/>
+      <c r="K18" s="7"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="19"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="18">
+      <c r="C19" s="21"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="20">
         <v>7</v>
       </c>
-      <c r="G19" s="20"/>
+      <c r="G19" s="22"/>
       <c r="H19" s="25">
         <f>H18/F19</f>
         <v>35714.285714285717</v>
       </c>
       <c r="I19" s="26"/>
-      <c r="J19" s="13">
+      <c r="J19" s="6">
         <f>G19*E19</f>
         <v>0</v>
       </c>
-      <c r="K19" s="14"/>
+      <c r="K19" s="7"/>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="41">
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="27">
         <f>H19+H16</f>
         <v>46968.285714285717</v>
       </c>
-      <c r="I20" s="42"/>
+      <c r="I20" s="28"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="32">
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="29">
         <f>H19/4+H17</f>
         <v>11742.071428571429</v>
       </c>
-      <c r="I21" s="40"/>
+      <c r="I21" s="30"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="33"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="37"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="69">
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="L12:M12"/>
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="J16:K16"/>
@@ -2451,46 +2455,32 @@
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="F16:G16"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="H13:I13"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="L12:M12"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="L10:M10"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="L6:M6"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="L3:M3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="L4" r:id="rId1" xr:uid="{18CD5E98-F315-49AA-9C2E-20515CC9BC5A}"/>

</xml_diff>